<commit_message>
Reverted doctors profiles in department specialities
</commit_message>
<xml_diff>
--- a/assets/excel/Staff_Doctor_Details(Responses).xlsx
+++ b/assets/excel/Staff_Doctor_Details(Responses).xlsx
@@ -1,19 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\NewSRMTrichy\assets\excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24240" windowHeight="12315"/>
   </bookViews>
   <sheets>
     <sheet name="Form Responses 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Form Responses 1'!$A$1:$AN$235</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -7215,7 +7213,7 @@
     <t>3/17/2025</t>
   </si>
   <si>
-    <t>Dental</t>
+    <t>Dentistry</t>
   </si>
 </sst>
 </file>
@@ -7291,7 +7289,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -7507,12 +7505,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="22" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -7676,6 +7689,9 @@
     </xf>
     <xf numFmtId="22" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -28957,7 +28973,7 @@
         <v>11</v>
       </c>
       <c r="Z199" s="9" t="s">
-        <v>553</v>
+        <v>270</v>
       </c>
       <c r="AA199" s="9" t="s">
         <v>553</v>
@@ -32157,7 +32173,7 @@
         <v>11</v>
       </c>
       <c r="Z229" s="31" t="s">
-        <v>1943</v>
+        <v>2153</v>
       </c>
       <c r="AA229" s="31" t="s">
         <v>2241</v>
@@ -32476,7 +32492,7 @@
       <c r="Y232" s="31" t="s">
         <v>199</v>
       </c>
-      <c r="Z232" s="31" t="s">
+      <c r="Z232" s="39" t="s">
         <v>2315</v>
       </c>
       <c r="AA232" s="31" t="s">
@@ -32794,7 +32810,7 @@
       <c r="Y235" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="Z235" s="47" t="s">
+      <c r="Z235" s="56" t="s">
         <v>2315</v>
       </c>
       <c r="AA235" s="47" t="s">

</xml_diff>